<commit_message>
HHR client template: remove leftover sample org/hotel/event placeholders
The template carried NCSL/Hyatt sample values in C2/C3/C4. The current code
overwrites these from the raw HHR, but clearing them is a safety net so a
report can never show stale placeholder hotel/event text if a header row is
ever missing from a source HHR.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/hhr_template.xlsx
+++ b/static/hhr_template.xlsx
@@ -1467,11 +1467,7 @@
         </is>
       </c>
       <c r="B2" s="142" t="n"/>
-      <c r="C2" s="111" t="inlineStr">
-        <is>
-          <t>NCSL</t>
-        </is>
-      </c>
+      <c r="C2" s="111" t="n"/>
       <c r="D2" s="140" t="n"/>
       <c r="E2" s="140" t="n"/>
       <c r="F2" s="140" t="n"/>
@@ -1490,11 +1486,7 @@
         </is>
       </c>
       <c r="B3" s="142" t="n"/>
-      <c r="C3" s="111" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hyatt Regency Washington on Capitol Hill </t>
-        </is>
-      </c>
+      <c r="C3" s="111" t="n"/>
       <c r="D3" s="140" t="n"/>
       <c r="E3" s="140" t="n"/>
       <c r="F3" s="140" t="n"/>
@@ -1513,11 +1505,7 @@
         </is>
       </c>
       <c r="B4" s="142" t="n"/>
-      <c r="C4" s="111" t="inlineStr">
-        <is>
-          <t>Capitol Connection</t>
-        </is>
-      </c>
+      <c r="C4" s="111" t="n"/>
       <c r="D4" s="140" t="n"/>
       <c r="E4" s="140" t="n"/>
       <c r="F4" s="140" t="n"/>
@@ -1984,8 +1972,8 @@
       </c>
       <c r="B19" s="150" t="n"/>
       <c r="C19" s="152" t="n"/>
-      <c r="D19" s="153" t="n"/>
-      <c r="E19" s="154" t="n"/>
+      <c r="D19" s="151" t="n"/>
+      <c r="E19" s="150" t="n"/>
     </row>
     <row r="20" ht="16" customFormat="1" customHeight="1" s="1">
       <c r="A20" s="146" t="inlineStr">
@@ -1995,8 +1983,8 @@
       </c>
       <c r="B20" s="150" t="n"/>
       <c r="C20" s="152" t="n"/>
-      <c r="D20" s="153" t="n"/>
-      <c r="E20" s="154" t="n"/>
+      <c r="D20" s="151" t="n"/>
+      <c r="E20" s="150" t="n"/>
     </row>
     <row r="21" ht="16" customFormat="1" customHeight="1" s="1">
       <c r="A21" s="146" t="inlineStr">
@@ -2006,8 +1994,8 @@
       </c>
       <c r="B21" s="150" t="n"/>
       <c r="C21" s="152" t="n"/>
-      <c r="D21" s="153" t="n"/>
-      <c r="E21" s="154" t="n"/>
+      <c r="D21" s="151" t="n"/>
+      <c r="E21" s="150" t="n"/>
     </row>
     <row r="22" ht="16" customHeight="1" s="67">
       <c r="A22" s="146" t="inlineStr">
@@ -2017,8 +2005,8 @@
       </c>
       <c r="B22" s="150" t="n"/>
       <c r="C22" s="152" t="n"/>
-      <c r="D22" s="153" t="n"/>
-      <c r="E22" s="154" t="n"/>
+      <c r="D22" s="151" t="n"/>
+      <c r="E22" s="150" t="n"/>
     </row>
     <row r="23" ht="30.25" customHeight="1" s="67"/>
     <row r="24" ht="39.25" customHeight="1" s="67"/>

</xml_diff>